<commit_message>
feat: primera versión del portal sin envío de correos
</commit_message>
<xml_diff>
--- a/portal-examenes-netec/specs/01-discovery/catalogo_examenes.xlsx
+++ b/portal-examenes-netec/specs/01-discovery/catalogo_examenes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dcbab197249526ff/trabajo/ProyectoTestingCenter/portal-examenes-netec/specs/01-discovery/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2CB724B2-3A6F-4FFB-B02B-08C19D98738B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{2CB724B2-3A6F-4FFB-B02B-08C19D98738B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49D5E879-50C2-44FE-AB46-980DAAFF27FD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F88B6EC9-A3B7-40C0-8491-2BBC6935E098}"/>
+    <workbookView minimized="1" xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11835" xr2:uid="{F88B6EC9-A3B7-40C0-8491-2BBC6935E098}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1393,6 +1393,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89918379-76E9-44E6-80A7-DD30EFE74B41}">
   <dimension ref="A2:G126"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="67.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">

</xml_diff>